<commit_message>
Run the carrot and mesclun schedules one bed past their caps
The shadow prices the memo leans on ($352.49 and $246.47) and the AVC
figures behind the at-a-loss answer had no cell behind them. Carrot bed 21
and mesclun bed 31 now sit in the schedules as Past cap rows, outside the
crossing counts and validation ranges, and every schedule carries
cumulative variable cost and AVC columns. The analysis cites the cells.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ARid7pzLFuChUL9uXc2AFK
</commit_message>
<xml_diff>
--- a/capabilities/marginal-analysis/model.xlsx
+++ b/capabilities/marginal-analysis/model.xlsx
@@ -357,10 +357,10 @@
     <t>Dip flag</t>
   </si>
   <si>
-    <t>CARROTS — standalone schedule (q = 0 to CAR_CAP)</t>
-  </si>
-  <si>
-    <t>MESCLUN — standalone schedule (q = 0 to MES_CAP)</t>
+    <t>CARROTS — standalone schedule (q = 0 to CAR_CAP, plus bed 21 past the cap: its P − MC is the cap's shadow price)</t>
+  </si>
+  <si>
+    <t>MESCLUN — standalone schedule (q = 0 to MES_CAP, plus bed 31 past the cap: its P − MC is the cap's shadow price)</t>
   </si>
   <si>
     <t>Standalone crossing points and the tomato dip</t>
@@ -2060,7 +2060,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:K96"/>
+  <dimension ref="A1:M96"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
@@ -2071,6 +2071,8 @@
     <col min="7" max="7" width="14" customWidth="1"/>
     <col min="8" max="10" width="13" customWidth="1"/>
     <col min="11" max="11" width="9" customWidth="1"/>
+    <col min="12" max="12" width="17" customWidth="1"/>
+    <col min="13" max="13" width="13" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="19" x14ac:dyDescent="0.25">
@@ -2093,7 +2095,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
         <v>67</v>
       </c>
@@ -2126,6 +2128,16 @@
       </c>
       <c r="K6" s="4" t="s">
         <v>77</v>
+      </c>
+      <c r="L6" s="4" t="inlineStr">
+        <is>
+          <t>Cumulative VC(q)</t>
+        </is>
+      </c>
+      <c r="M6" s="4" t="inlineStr">
+        <is>
+          <t>AVC(q)</t>
+        </is>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
@@ -2146,7 +2158,7 @@
       <c r="J7" s="16"/>
       <c r="K7" s="16"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" s="14">
         <v>1</v>
       </c>
@@ -2190,8 +2202,16 @@
         <f t="shared" ref="K8:K27" si="8">IF(A8&lt;2,0,IF(G8&lt;G7,1,0))</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L8" s="17">
+        <f>SUM($G$8:G8)</f>
+        <v>4317.5</v>
+      </c>
+      <c r="M8" s="17">
+        <f>L8/A8</f>
+        <v>4317.5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" s="14">
         <v>2</v>
       </c>
@@ -2235,8 +2255,16 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L9" s="17">
+        <f>SUM($G$8:G9)</f>
+        <v>9322.5</v>
+      </c>
+      <c r="M9" s="17">
+        <f>L9/A9</f>
+        <v>4661.25</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" s="14">
         <v>3</v>
       </c>
@@ -2280,8 +2308,16 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L10" s="17">
+        <f>SUM($G$8:G10)</f>
+        <v>15118.125000000004</v>
+      </c>
+      <c r="M10" s="17">
+        <f>L10/A10</f>
+        <v>5039.375000000001</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" s="14">
         <v>4</v>
       </c>
@@ -2325,8 +2361,16 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L11" s="17">
+        <f>SUM($G$8:G11)</f>
+        <v>21821.250000000004</v>
+      </c>
+      <c r="M11" s="17">
+        <f>L11/A11</f>
+        <v>5455.312500000001</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" s="14">
         <v>5</v>
       </c>
@@ -2370,8 +2414,16 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L12" s="17">
+        <f>SUM($G$8:G12)</f>
+        <v>29482.109375000004</v>
+      </c>
+      <c r="M12" s="17">
+        <f>L12/A12</f>
+        <v>5896.421875000001</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A13" s="14">
         <v>6</v>
       </c>
@@ -2415,8 +2467,16 @@
         <f t="shared" si="8"/>
         <v>1</v>
       </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L13" s="17">
+        <f>SUM($G$8:G13)</f>
+        <v>34388.38437500001</v>
+      </c>
+      <c r="M13" s="17">
+        <f>L13/A13</f>
+        <v>5731.3973958333345</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14" s="14">
         <v>7</v>
       </c>
@@ -2460,8 +2520,16 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L14" s="17">
+        <f>SUM($G$8:G14)</f>
+        <v>39974.09328125001</v>
+      </c>
+      <c r="M14" s="17">
+        <f>L14/A14</f>
+        <v>5710.5847544642875</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A15" s="14">
         <v>8</v>
       </c>
@@ -2505,8 +2573,16 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L15" s="17">
+        <f>SUM($G$8:G15)</f>
+        <v>46334.86012500002</v>
+      </c>
+      <c r="M15" s="17">
+        <f>L15/A15</f>
+        <v>5791.857515625003</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A16" s="14">
         <v>9</v>
       </c>
@@ -2550,8 +2626,16 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L16" s="17">
+        <f>SUM($G$8:G16)</f>
+        <v>53578.63940468753</v>
+      </c>
+      <c r="M16" s="17">
+        <f>L16/A16</f>
+        <v>5953.182156076392</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A17" s="14">
         <v>10</v>
       </c>
@@ -2595,8 +2679,16 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L17" s="17">
+        <f>SUM($G$8:G17)</f>
+        <v>61827.22593906253</v>
+      </c>
+      <c r="M17" s="17">
+        <f>L17/A17</f>
+        <v>6182.722593906254</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A18" s="14">
         <v>11</v>
       </c>
@@ -2640,8 +2732,16 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L18" s="17">
+        <f>SUM($G$8:G18)</f>
+        <v>71217.94338626566</v>
+      </c>
+      <c r="M18" s="17">
+        <f>L18/A18</f>
+        <v>6474.358489660514</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A19" s="14">
         <v>12</v>
       </c>
@@ -2685,8 +2785,16 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L19" s="17">
+        <f>SUM($G$8:G19)</f>
+        <v>81905.5320635188</v>
+      </c>
+      <c r="M19" s="17">
+        <f>L19/A19</f>
+        <v>6825.461005293233</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A20" s="14">
         <v>13</v>
       </c>
@@ -2730,8 +2838,16 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L20" s="17">
+        <f>SUM($G$8:G20)</f>
+        <v>94064.2590423599</v>
+      </c>
+      <c r="M20" s="17">
+        <f>L20/A20</f>
+        <v>7235.712234027685</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A21" s="14">
         <v>14</v>
       </c>
@@ -2775,8 +2891,16 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L21" s="17">
+        <f>SUM($G$8:G21)</f>
+        <v>107890.27609633406</v>
+      </c>
+      <c r="M21" s="17">
+        <f>L21/A21</f>
+        <v>7706.44829259529</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A22" s="14">
         <v>15</v>
       </c>
@@ -2820,8 +2944,16 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L22" s="17">
+        <f>SUM($G$8:G22)</f>
+        <v>123604.25397067943</v>
+      </c>
+      <c r="M22" s="17">
+        <f>L22/A22</f>
+        <v>8240.283598045296</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A23" s="14">
         <v>16</v>
       </c>
@@ -2865,8 +2997,16 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L23" s="17">
+        <f>SUM($G$8:G23)</f>
+        <v>141454.32465893053</v>
+      </c>
+      <c r="M23" s="17">
+        <f>L23/A23</f>
+        <v>8840.895291183158</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A24" s="14">
         <v>17</v>
       </c>
@@ -2910,8 +3050,16 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L24" s="17">
+        <f>SUM($G$8:G24)</f>
+        <v>161719.36694512508</v>
+      </c>
+      <c r="M24" s="17">
+        <f>L24/A24</f>
+        <v>9512.903937948533</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A25" s="14">
         <v>18</v>
       </c>
@@ -2955,8 +3103,16 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L25" s="17">
+        <f>SUM($G$8:G25)</f>
+        <v>184712.6744419692</v>
+      </c>
+      <c r="M25" s="17">
+        <f>L25/A25</f>
+        <v>10261.815246776066</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A26" s="14">
         <v>19</v>
       </c>
@@ -3000,8 +3156,16 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L26" s="17">
+        <f>SUM($G$8:G26)</f>
+        <v>210786.04976873094</v>
+      </c>
+      <c r="M26" s="17">
+        <f>L26/A26</f>
+        <v>11094.002619406892</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A27" s="14">
         <v>20</v>
       </c>
@@ -3045,13 +3209,21 @@
         <f t="shared" si="8"/>
         <v>0</v>
       </c>
+      <c r="L27" s="17">
+        <f>SUM($G$8:G27)</f>
+        <v>240334.3734164253</v>
+      </c>
+      <c r="M27" s="17">
+        <f>L27/A27</f>
+        <v>12016.718670821265</v>
+      </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A30" s="3" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A31" s="4" t="s">
         <v>67</v>
       </c>
@@ -3084,6 +3256,16 @@
       </c>
       <c r="K31" s="4" t="s">
         <v>77</v>
+      </c>
+      <c r="L31" s="4" t="inlineStr">
+        <is>
+          <t>Cumulative VC(q)</t>
+        </is>
+      </c>
+      <c r="M31" s="4" t="inlineStr">
+        <is>
+          <t>AVC(q)</t>
+        </is>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.2">
@@ -3104,7 +3286,7 @@
       <c r="J32" s="16"/>
       <c r="K32" s="16"/>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A33" s="14">
         <v>1</v>
       </c>
@@ -3148,8 +3330,16 @@
         <f t="shared" ref="K33:K52" si="17">IF(A33&lt;2,0,IF(G33&lt;G32,1,0))</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L33" s="17">
+        <f>SUM($G$33:G33)</f>
+        <v>1507.7083333333333</v>
+      </c>
+      <c r="M33" s="17">
+        <f>L33/A33</f>
+        <v>1507.7083333333333</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A34" s="14">
         <v>2</v>
       </c>
@@ -3193,8 +3383,16 @@
         <f t="shared" si="17"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L34" s="17">
+        <f>SUM($G$33:G34)</f>
+        <v>3068.802083333333</v>
+      </c>
+      <c r="M34" s="17">
+        <f>L34/A34</f>
+        <v>1534.4010416666665</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A35" s="14">
         <v>3</v>
       </c>
@@ -3238,8 +3436,16 @@
         <f t="shared" si="17"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L35" s="17">
+        <f>SUM($G$33:G35)</f>
+        <v>4685.283203124998</v>
+      </c>
+      <c r="M35" s="17">
+        <f>L35/A35</f>
+        <v>1561.7610677083328</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A36" s="14">
         <v>4</v>
       </c>
@@ -3283,8 +3489,16 @@
         <f t="shared" si="17"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L36" s="17">
+        <f>SUM($G$33:G36)</f>
+        <v>6359.220377604164</v>
+      </c>
+      <c r="M36" s="17">
+        <f>L36/A36</f>
+        <v>1589.805094401041</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A37" s="14">
         <v>5</v>
       </c>
@@ -3328,8 +3542,16 @@
         <f t="shared" si="17"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L37" s="17">
+        <f>SUM($G$33:G37)</f>
+        <v>8092.751108805335</v>
+      </c>
+      <c r="M37" s="17">
+        <f>L37/A37</f>
+        <v>1618.550221761067</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A38" s="14">
         <v>6</v>
       </c>
@@ -3373,8 +3595,16 @@
         <f t="shared" si="17"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L38" s="17">
+        <f>SUM($G$33:G38)</f>
+        <v>9888.083863830561</v>
+      </c>
+      <c r="M38" s="17">
+        <f>L38/A38</f>
+        <v>1648.0139773050935</v>
+      </c>
+    </row>
+    <row r="39" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A39" s="14">
         <v>7</v>
       </c>
@@ -3418,8 +3648,16 @@
         <f t="shared" si="17"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L39" s="17">
+        <f>SUM($G$33:G39)</f>
+        <v>11747.500287164048</v>
+      </c>
+      <c r="M39" s="17">
+        <f>L39/A39</f>
+        <v>1678.2143267377212</v>
+      </c>
+    </row>
+    <row r="40" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A40" s="14">
         <v>8</v>
       </c>
@@ -3463,8 +3701,16 @@
         <f t="shared" si="17"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L40" s="17">
+        <f>SUM($G$33:G40)</f>
+        <v>13673.35747924931</v>
+      </c>
+      <c r="M40" s="17">
+        <f>L40/A40</f>
+        <v>1709.1696849061636</v>
+      </c>
+    </row>
+    <row r="41" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A41" s="14">
         <v>9</v>
       </c>
@@ -3508,8 +3754,16 @@
         <f t="shared" si="17"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L41" s="17">
+        <f>SUM($G$33:G41)</f>
+        <v>15668.09034325936</v>
+      </c>
+      <c r="M41" s="17">
+        <f>L41/A41</f>
+        <v>1740.8989270288178</v>
+      </c>
+    </row>
+    <row r="42" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A42" s="14">
         <v>10</v>
       </c>
@@ -3553,8 +3807,16 @@
         <f t="shared" si="17"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L42" s="17">
+        <f>SUM($G$33:G42)</f>
+        <v>17734.21400204538</v>
+      </c>
+      <c r="M42" s="17">
+        <f>L42/A42</f>
+        <v>1773.421400204538</v>
+      </c>
+    </row>
+    <row r="43" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A43" s="14">
         <v>11</v>
       </c>
@@ -3598,8 +3860,16 @@
         <f t="shared" si="17"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L43" s="17">
+        <f>SUM($G$33:G43)</f>
+        <v>19874.32628730617</v>
+      </c>
+      <c r="M43" s="17">
+        <f>L43/A43</f>
+        <v>1806.7569352096516</v>
+      </c>
+    </row>
+    <row r="44" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A44" s="14">
         <v>12</v>
       </c>
@@ -3643,8 +3913,16 @@
         <f t="shared" si="17"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L44" s="17">
+        <f>SUM($G$33:G44)</f>
+        <v>22091.110303078713</v>
+      </c>
+      <c r="M44" s="17">
+        <f>L44/A44</f>
+        <v>1840.9258585898926</v>
+      </c>
+    </row>
+    <row r="45" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A45" s="14">
         <v>13</v>
       </c>
@@ -3688,8 +3966,16 @@
         <f t="shared" si="17"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L45" s="17">
+        <f>SUM($G$33:G45)</f>
+        <v>24387.337065710315</v>
+      </c>
+      <c r="M45" s="17">
+        <f>L45/A45</f>
+        <v>1875.9490050546397</v>
+      </c>
+    </row>
+    <row r="46" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A46" s="14">
         <v>14</v>
       </c>
@@ -3733,8 +4019,16 @@
         <f t="shared" si="17"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L46" s="17">
+        <f>SUM($G$33:G46)</f>
+        <v>26765.86822253408</v>
+      </c>
+      <c r="M46" s="17">
+        <f>L46/A46</f>
+        <v>1911.8477301810058</v>
+      </c>
+    </row>
+    <row r="47" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A47" s="14">
         <v>15</v>
       </c>
@@ -3778,8 +4072,16 @@
         <f t="shared" si="17"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L47" s="17">
+        <f>SUM($G$33:G47)</f>
+        <v>29229.65885153296</v>
+      </c>
+      <c r="M47" s="17">
+        <f>L47/A47</f>
+        <v>1948.6439234355307</v>
+      </c>
+    </row>
+    <row r="48" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A48" s="14">
         <v>16</v>
       </c>
@@ -3823,8 +4125,16 @@
         <f t="shared" si="17"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L48" s="17">
+        <f>SUM($G$33:G48)</f>
+        <v>31781.7603443427</v>
+      </c>
+      <c r="M48" s="17">
+        <f>L48/A48</f>
+        <v>1986.3600215214187</v>
+      </c>
+    </row>
+    <row r="49" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A49" s="14">
         <v>17</v>
       </c>
@@ -3868,8 +4178,16 @@
         <f t="shared" si="17"/>
         <v>1</v>
       </c>
-    </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L49" s="17">
+        <f>SUM($G$33:G49)</f>
+        <v>33452.66168750536</v>
+      </c>
+      <c r="M49" s="17">
+        <f>L49/A49</f>
+        <v>1967.8036286767858</v>
+      </c>
+    </row>
+    <row r="50" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A50" s="14">
         <v>18</v>
       </c>
@@ -3913,8 +4231,16 @@
         <f t="shared" si="17"/>
         <v>1</v>
       </c>
-    </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L50" s="17">
+        <f>SUM($G$33:G50)</f>
+        <v>35041.80047849846</v>
+      </c>
+      <c r="M50" s="17">
+        <f>L50/A50</f>
+        <v>1946.7666932499144</v>
+      </c>
+    </row>
+    <row r="51" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A51" s="14">
         <v>19</v>
       </c>
@@ -3958,8 +4284,16 @@
         <f t="shared" si="17"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L51" s="17">
+        <f>SUM($G$33:G51)</f>
+        <v>36679.97579548653</v>
+      </c>
+      <c r="M51" s="17">
+        <f>L51/A51</f>
+        <v>1930.525041867712</v>
+      </c>
+    </row>
+    <row r="52" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A52" s="14">
         <v>20</v>
       </c>
@@ -4003,13 +4337,71 @@
         <f t="shared" si="17"/>
         <v>0</v>
       </c>
+      <c r="L52" s="17">
+        <f>SUM($G$33:G52)</f>
+        <v>38368.921253024935</v>
+      </c>
+      <c r="M52" s="17">
+        <f>L52/A52</f>
+        <v>1918.4460626512468</v>
+      </c>
+    </row>
+    <row r="53" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A53" s="14">
+        <v>21</v>
+      </c>
+      <c r="B53" s="15">
+        <f>A53*CAR_HPB*WEEKS*(1+CAR_DIM)^A53</f>
+        <v>1058.136566317522</v>
+      </c>
+      <c r="C53" s="15">
+        <f>B53-B52</f>
+        <v>74.96670214328549</v>
+      </c>
+      <c r="D53" s="15">
+        <f>MAX(0,MIN(C53,PERM_HOURS-B52))</f>
+        <v>0.0</v>
+      </c>
+      <c r="E53" s="15">
+        <f>C53-D53</f>
+        <v>74.96670214328549</v>
+      </c>
+      <c r="F53" s="17">
+        <f>CAR_FERT</f>
+        <v>440.0</v>
+      </c>
+      <c r="G53" s="17">
+        <f>D53*PERM_RATE+E53*TEMP_RATE+F53</f>
+        <v>1741.5052455431507</v>
+      </c>
+      <c r="H53" s="17">
+        <f>CAR_PRICE</f>
+        <v>2094.0</v>
+      </c>
+      <c r="I53" s="17">
+        <f>H53-G53</f>
+        <v>352.49475445684925</v>
+      </c>
+      <c r="J53" s="18" t="inlineStr">
+        <is>
+          <t>Past cap</t>
+        </is>
+      </c>
+      <c r="L53" s="17">
+        <f>SUM($G$33:G53)</f>
+        <v>40110.426498568086</v>
+      </c>
+      <c r="M53" s="17">
+        <f>L53/A53</f>
+        <v>1910.0203094556232</v>
+      </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A55" s="3" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A56" s="4" t="s">
         <v>67</v>
       </c>
@@ -4042,6 +4434,16 @@
       </c>
       <c r="K56" s="4" t="s">
         <v>77</v>
+      </c>
+      <c r="L56" s="4" t="inlineStr">
+        <is>
+          <t>Cumulative VC(q)</t>
+        </is>
+      </c>
+      <c r="M56" s="4" t="inlineStr">
+        <is>
+          <t>AVC(q)</t>
+        </is>
       </c>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.2">
@@ -4062,7 +4464,7 @@
       <c r="J57" s="16"/>
       <c r="K57" s="16"/>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A58" s="14">
         <v>1</v>
       </c>
@@ -4106,8 +4508,16 @@
         <f t="shared" ref="K58:K87" si="26">IF(A58&lt;2,0,IF(G58&lt;G57,1,0))</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L58" s="17">
+        <f>SUM($G$58:G58)</f>
+        <v>2462.03125</v>
+      </c>
+      <c r="M58" s="17">
+        <f>L58/A58</f>
+        <v>2462.03125</v>
+      </c>
+    </row>
+    <row r="59" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A59" s="14">
         <v>2</v>
       </c>
@@ -4151,8 +4561,16 @@
         <f t="shared" si="26"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L59" s="17">
+        <f>SUM($G$58:G59)</f>
+        <v>4963.61328125</v>
+      </c>
+      <c r="M59" s="17">
+        <f>L59/A59</f>
+        <v>2481.806640625</v>
+      </c>
+    </row>
+    <row r="60" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A60" s="14">
         <v>3</v>
       </c>
@@ -4196,8 +4614,16 @@
         <f t="shared" si="26"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L60" s="17">
+        <f>SUM($G$58:G60)</f>
+        <v>7505.487670898437</v>
+      </c>
+      <c r="M60" s="17">
+        <f>L60/A60</f>
+        <v>2501.829223632812</v>
+      </c>
+    </row>
+    <row r="61" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A61" s="14">
         <v>4</v>
       </c>
@@ -4241,8 +4667,16 @@
         <f t="shared" si="26"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L61" s="17">
+        <f>SUM($G$58:G61)</f>
+        <v>10088.408355712889</v>
+      </c>
+      <c r="M61" s="17">
+        <f>L61/A61</f>
+        <v>2522.102088928222</v>
+      </c>
+    </row>
+    <row r="62" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A62" s="14">
         <v>5</v>
       </c>
@@ -4286,8 +4720,16 @@
         <f t="shared" si="26"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L62" s="17">
+        <f>SUM($G$58:G62)</f>
+        <v>12713.141825199125</v>
+      </c>
+      <c r="M62" s="17">
+        <f>L62/A62</f>
+        <v>2542.628365039825</v>
+      </c>
+    </row>
+    <row r="63" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A63" s="14">
         <v>6</v>
       </c>
@@ -4331,8 +4773,16 @@
         <f t="shared" si="26"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L63" s="17">
+        <f>SUM($G$58:G63)</f>
+        <v>15380.467317616934</v>
+      </c>
+      <c r="M63" s="17">
+        <f>L63/A63</f>
+        <v>2563.4112196028223</v>
+      </c>
+    </row>
+    <row r="64" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A64" s="14">
         <v>7</v>
       </c>
@@ -4376,8 +4826,16 @@
         <f t="shared" si="26"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L64" s="17">
+        <f>SUM($G$58:G64)</f>
+        <v>18091.177018935006</v>
+      </c>
+      <c r="M64" s="17">
+        <f>L64/A64</f>
+        <v>2584.453859847858</v>
+      </c>
+    </row>
+    <row r="65" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A65" s="14">
         <v>8</v>
       </c>
@@ -4421,8 +4879,16 @@
         <f t="shared" si="26"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L65" s="17">
+        <f>SUM($G$58:G65)</f>
+        <v>20846.07626476765</v>
+      </c>
+      <c r="M65" s="17">
+        <f>L65/A65</f>
+        <v>2605.759533095956</v>
+      </c>
+    </row>
+    <row r="66" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A66" s="14">
         <v>9</v>
       </c>
@@ -4466,8 +4932,16 @@
         <f t="shared" si="26"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L66" s="17">
+        <f>SUM($G$58:G66)</f>
+        <v>23645.9837453369</v>
+      </c>
+      <c r="M66" s="17">
+        <f>L66/A66</f>
+        <v>2627.3315272596556</v>
+      </c>
+    </row>
+    <row r="67" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A67" s="14">
         <v>10</v>
       </c>
@@ -4511,8 +4985,16 @@
         <f t="shared" si="26"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L67" s="17">
+        <f>SUM($G$58:G67)</f>
+        <v>26491.73171350401</v>
+      </c>
+      <c r="M67" s="17">
+        <f>L67/A67</f>
+        <v>2649.173171350401</v>
+      </c>
+    </row>
+    <row r="68" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A68" s="14">
         <v>11</v>
       </c>
@@ -4556,8 +5038,16 @@
         <f t="shared" si="26"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L68" s="17">
+        <f>SUM($G$58:G68)</f>
+        <v>29384.16619591509</v>
+      </c>
+      <c r="M68" s="17">
+        <f>L68/A68</f>
+        <v>2671.287835992281</v>
+      </c>
+    </row>
+    <row r="69" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A69" s="14">
         <v>12</v>
       </c>
@@ -4601,8 +5091,16 @@
         <f t="shared" si="26"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L69" s="17">
+        <f>SUM($G$58:G69)</f>
+        <v>32324.147207306214</v>
+      </c>
+      <c r="M69" s="17">
+        <f>L69/A69</f>
+        <v>2693.6789339421844</v>
+      </c>
+    </row>
+    <row r="70" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A70" s="14">
         <v>13</v>
       </c>
@@ -4646,8 +5144,16 @@
         <f t="shared" si="26"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L70" s="17">
+        <f>SUM($G$58:G70)</f>
+        <v>35312.548968014</v>
+      </c>
+      <c r="M70" s="17">
+        <f>L70/A70</f>
+        <v>2716.3499206164615</v>
+      </c>
+    </row>
+    <row r="71" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A71" s="14">
         <v>14</v>
       </c>
@@ -4691,8 +5197,16 @@
         <f t="shared" si="26"/>
         <v>1</v>
       </c>
-    </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L71" s="17">
+        <f>SUM($G$58:G71)</f>
+        <v>37835.13006236917</v>
+      </c>
+      <c r="M71" s="17">
+        <f>L71/A71</f>
+        <v>2702.5092901692265</v>
+      </c>
+    </row>
+    <row r="72" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A72" s="14">
         <v>15</v>
       </c>
@@ -4736,8 +5250,16 @@
         <f t="shared" si="26"/>
         <v>1</v>
       </c>
-    </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L72" s="17">
+        <f>SUM($G$58:G72)</f>
+        <v>39819.091987302265</v>
+      </c>
+      <c r="M72" s="17">
+        <f>L72/A72</f>
+        <v>2654.606132486818</v>
+      </c>
+    </row>
+    <row r="73" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A73" s="14">
         <v>16</v>
       </c>
@@ -4781,8 +5303,16 @@
         <f t="shared" si="26"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L73" s="17">
+        <f>SUM($G$58:G73)</f>
+        <v>41828.61934628645</v>
+      </c>
+      <c r="M73" s="17">
+        <f>L73/A73</f>
+        <v>2614.288709142903</v>
+      </c>
+    </row>
+    <row r="74" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A74" s="14">
         <v>17</v>
       </c>
@@ -4826,8 +5356,16 @@
         <f t="shared" si="26"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L74" s="17">
+        <f>SUM($G$58:G74)</f>
+        <v>43864.17878112222</v>
+      </c>
+      <c r="M74" s="17">
+        <f>L74/A74</f>
+        <v>2580.245810654248</v>
+      </c>
+    </row>
+    <row r="75" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A75" s="14">
         <v>18</v>
       </c>
@@ -4871,8 +5409,16 @@
         <f t="shared" si="26"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L75" s="17">
+        <f>SUM($G$58:G75)</f>
+        <v>45926.244605056025</v>
+      </c>
+      <c r="M75" s="17">
+        <f>L75/A75</f>
+        <v>2551.4580336142235</v>
+      </c>
+    </row>
+    <row r="76" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A76" s="14">
         <v>19</v>
       </c>
@@ -4916,8 +5462,16 @@
         <f t="shared" si="26"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L76" s="17">
+        <f>SUM($G$58:G76)</f>
+        <v>48015.29892165363</v>
+      </c>
+      <c r="M76" s="17">
+        <f>L76/A76</f>
+        <v>2527.1209958765066</v>
+      </c>
+    </row>
+    <row r="77" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A77" s="14">
         <v>20</v>
       </c>
@@ -4961,8 +5515,16 @@
         <f t="shared" si="26"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L77" s="17">
+        <f>SUM($G$58:G77)</f>
+        <v>50131.83174544663</v>
+      </c>
+      <c r="M77" s="17">
+        <f>L77/A77</f>
+        <v>2506.5915872723317</v>
+      </c>
+    </row>
+    <row r="78" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A78" s="14">
         <v>21</v>
       </c>
@@ -5006,8 +5568,16 @@
         <f t="shared" si="26"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L78" s="17">
+        <f>SUM($G$58:G78)</f>
+        <v>52276.34112437795</v>
+      </c>
+      <c r="M78" s="17">
+        <f>L78/A78</f>
+        <v>2489.349577351331</v>
+      </c>
+    </row>
+    <row r="79" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A79" s="14">
         <v>22</v>
       </c>
@@ -5051,8 +5621,16 @@
         <f t="shared" si="26"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L79" s="17">
+        <f>SUM($G$58:G79)</f>
+        <v>54449.333264072324</v>
+      </c>
+      <c r="M79" s="17">
+        <f>L79/A79</f>
+        <v>2474.9696938214693</v>
+      </c>
+    </row>
+    <row r="80" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A80" s="14">
         <v>23</v>
       </c>
@@ -5096,8 +5674,16 @@
         <f t="shared" si="26"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L80" s="17">
+        <f>SUM($G$58:G80)</f>
+        <v>56651.32265395837</v>
+      </c>
+      <c r="M80" s="17">
+        <f>L80/A80</f>
+        <v>2463.1009849547117</v>
+      </c>
+    </row>
+    <row r="81" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A81" s="14">
         <v>24</v>
       </c>
@@ -5141,8 +5727,16 @@
         <f t="shared" si="26"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L81" s="17">
+        <f>SUM($G$58:G81)</f>
+        <v>58882.83219526906</v>
+      </c>
+      <c r="M81" s="17">
+        <f>L81/A81</f>
+        <v>2453.4513414695443</v>
+      </c>
+    </row>
+    <row r="82" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A82" s="14">
         <v>25</v>
       </c>
@@ -5186,8 +5780,16 @@
         <f t="shared" si="26"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L82" s="17">
+        <f>SUM($G$58:G82)</f>
+        <v>61144.39333094784</v>
+      </c>
+      <c r="M82" s="17">
+        <f>L82/A82</f>
+        <v>2445.7757332379133</v>
+      </c>
+    </row>
+    <row r="83" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A83" s="14">
         <v>26</v>
       </c>
@@ -5231,8 +5833,16 @@
         <f t="shared" si="26"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L83" s="17">
+        <f>SUM($G$58:G83)</f>
+        <v>63436.54617748807</v>
+      </c>
+      <c r="M83" s="17">
+        <f>L83/A83</f>
+        <v>2439.867160672618</v>
+      </c>
+    </row>
+    <row r="84" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A84" s="14">
         <v>27</v>
       </c>
@@ -5276,8 +5886,16 @@
         <f t="shared" si="26"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L84" s="17">
+        <f>SUM($G$58:G84)</f>
+        <v>65759.83965873385</v>
+      </c>
+      <c r="M84" s="17">
+        <f>L84/A84</f>
+        <v>2435.5496169901426</v>
+      </c>
+    </row>
+    <row r="85" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A85" s="14">
         <v>28</v>
       </c>
@@ -5321,8 +5939,16 @@
         <f t="shared" si="26"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L85" s="17">
+        <f>SUM($G$58:G85)</f>
+        <v>68114.83164167053</v>
+      </c>
+      <c r="M85" s="17">
+        <f>L85/A85</f>
+        <v>2432.6725586310904</v>
+      </c>
+    </row>
+    <row r="86" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A86" s="14">
         <v>29</v>
       </c>
@@ -5366,8 +5992,16 @@
         <f t="shared" si="26"/>
         <v>0</v>
       </c>
-    </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L86" s="17">
+        <f>SUM($G$58:G86)</f>
+        <v>70502.08907423395</v>
+      </c>
+      <c r="M86" s="17">
+        <f>L86/A86</f>
+        <v>2431.1065198011706</v>
+      </c>
+    </row>
+    <row r="87" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A87" s="14">
         <v>30</v>
       </c>
@@ -5410,6 +6044,64 @@
       <c r="K87" s="19">
         <f t="shared" si="26"/>
         <v>0</v>
+      </c>
+      <c r="L87" s="17">
+        <f>SUM($G$58:G87)</f>
+        <v>72922.18812516746</v>
+      </c>
+      <c r="M87" s="17">
+        <f>L87/A87</f>
+        <v>2430.7396041722486</v>
+      </c>
+    </row>
+    <row r="88" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A88" s="14">
+        <v>31</v>
+      </c>
+      <c r="B88" s="15">
+        <f>A88*MES_HPB*WEEKS*(1+MES_DIM)^A88</f>
+        <v>2050.313145175093</v>
+      </c>
+      <c r="C88" s="15">
+        <f>B88-B87</f>
+        <v>90.63510916544624</v>
+      </c>
+      <c r="D88" s="15">
+        <f>MAX(0,MIN(C88,PERM_HOURS-B87))</f>
+        <v>0.0</v>
+      </c>
+      <c r="E88" s="15">
+        <f>C88-D88</f>
+        <v>90.63510916544624</v>
+      </c>
+      <c r="F88" s="17">
+        <f>MES_FERT</f>
+        <v>880.0</v>
+      </c>
+      <c r="G88" s="17">
+        <f>D88*PERM_RATE+E88*TEMP_RATE+F88</f>
+        <v>2453.526200788997</v>
+      </c>
+      <c r="H88" s="17">
+        <f>MES_PRICE</f>
+        <v>2700.0</v>
+      </c>
+      <c r="I88" s="17">
+        <f>H88-G88</f>
+        <v>246.4737992110031</v>
+      </c>
+      <c r="J88" s="18" t="inlineStr">
+        <is>
+          <t>Past cap</t>
+        </is>
+      </c>
+      <c r="L88" s="17">
+        <f>SUM($G$58:G88)</f>
+        <v>75375.71432595646</v>
+      </c>
+      <c r="M88" s="17">
+        <f>L88/A88</f>
+        <v>2431.474655676015</v>
       </c>
     </row>
     <row r="90" spans="1:11" x14ac:dyDescent="0.2">

</xml_diff>